<commit_message>
feat: add candidate research function classification with confidence and evidence
</commit_message>
<xml_diff>
--- a/assets/templates/candidate_import_template.xlsx
+++ b/assets/templates/candidate_import_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="候选人" sheetId="1" r:id="Rbb31009bc7aa461c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" r:id="R6d28a9a1c4c542f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="候选人" sheetId="1" r:id="R433805021e6e4237"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" r:id="Rf9618d9b7b1e4c6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3438,7 +3438,7 @@
         <x:v>2 · 一行一人</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
-        <x:v>在“候选人”表第一行保留列名，从第二行开始填写；每批最多 1,000 人、文件不超过 10 MB。</x:v>
+        <x:v>在“候选人”表第一行保留列名，从第二行开始填写；不设候选人人数上限，文件不超过 10 MB。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="55" customHeight="1">

</xml_diff>